<commit_message>
feat: add task comment options dialog
</commit_message>
<xml_diff>
--- a/outputs/quarter_planning_step1.xlsx
+++ b/outputs/quarter_planning_step1.xlsx
@@ -11,13 +11,14 @@
     <sheet sheetId="5" name="04_Квартальный план" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="99_Справочники" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="100_Шаблон экспресс оценки" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="101_Списки" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4596" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4713" uniqueCount="296">
   <si>
     <t>Настройки квартального планирования</t>
   </si>
@@ -355,6 +356,9 @@
     <t>QA</t>
   </si>
   <si>
+    <t>+</t>
+  </si>
+  <si>
     <t>Личный кабинет</t>
   </si>
   <si>
@@ -451,9 +455,6 @@
     <t>Баланс</t>
   </si>
   <si>
-    <t>+</t>
-  </si>
-  <si>
     <t>\</t>
   </si>
   <si>
@@ -857,6 +858,54 @@
   </si>
   <si>
     <t>[2] ЖЦ заявки</t>
+  </si>
+  <si>
+    <t>Списки</t>
+  </si>
+  <si>
+    <t>Артефакты</t>
+  </si>
+  <si>
+    <t>Смежники</t>
+  </si>
+  <si>
+    <t>БТ</t>
+  </si>
+  <si>
+    <t>Echo</t>
+  </si>
+  <si>
+    <t>Макеты</t>
+  </si>
+  <si>
+    <t>Sierra</t>
+  </si>
+  <si>
+    <t>ОТАР</t>
+  </si>
+  <si>
+    <t>Bravo</t>
+  </si>
+  <si>
+    <t>ПСИ ИБ</t>
+  </si>
+  <si>
+    <t>Foxtrot</t>
+  </si>
+  <si>
+    <t>Uniform</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Ф1</t>
+  </si>
+  <si>
+    <t>ЕСК</t>
+  </si>
+  <si>
+    <t>Тесса</t>
   </si>
 </sst>
 </file>
@@ -1518,6 +1567,30 @@
 </table>
 </file>
 
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" name="tblTaskCommentArtifacts" displayName="tblTaskCommentArtifacts" ref="A3:A7" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A3:A7">
+    <filterColumn colId="0" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="1">
+    <tableColumn id="1" name="Артефакты" totalsRowLabel="Total"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" name="tblTaskCommentAdjacentTeams" displayName="tblTaskCommentAdjacentTeams" ref="C3:C12" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="C3:C12">
+    <filterColumn colId="0" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="1">
+    <tableColumn id="1" name="Смежники" totalsRowLabel="Total"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" name="tblTeamMembers" displayName="tblTeamMembers" ref="A23:L43" totalsRowShown="0" headerRowCount="1">
   <autoFilter ref="A23:L43">
@@ -4101,7 +4174,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M103"/>
+  <dimension ref="A1:N103"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="5.857142857142857" customWidth="1"/>
@@ -4113,6 +4186,7 @@
     <col min="8" max="11" width="7.285714285714286" customWidth="1"/>
     <col min="12" max="12" width="73.42857142857143" customWidth="1"/>
     <col min="13" max="13" width="19.285714285714285" customWidth="1"/>
+    <col min="14" max="14" width="5.857142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:11" x14ac:dyDescent="0.25">
@@ -4156,7 +4230,7 @@
         <f>SUM(K4:K103)</f>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>101</v>
       </c>
@@ -4196,8 +4270,11 @@
       <c r="M3" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N3" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
         <v>101</v>
       </c>
@@ -4208,16 +4285,16 @@
         <v>10</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H4" s="29">
         <v>3</v>
@@ -4237,8 +4314,11 @@
       <c r="M4" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N4" s="27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
         <v>101</v>
       </c>
@@ -4249,13 +4329,13 @@
         <v>20</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>20</v>
@@ -4278,8 +4358,11 @@
       <c r="M5" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N5" s="27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
         <v>101</v>
       </c>
@@ -4290,13 +4373,13 @@
         <v>30</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>20</v>
@@ -4319,8 +4402,11 @@
       <c r="M6" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N6" s="27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
         <v>101</v>
       </c>
@@ -4331,13 +4417,13 @@
         <v>40</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>20</v>
@@ -4360,8 +4446,11 @@
       <c r="M7" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N7" s="27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
         <v>101</v>
       </c>
@@ -4372,13 +4461,13 @@
         <v>50</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>20</v>
@@ -4401,8 +4490,11 @@
       <c r="M8" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N8" s="27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
         <v>101</v>
       </c>
@@ -4413,13 +4505,13 @@
         <v>60</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>20</v>
@@ -4442,8 +4534,11 @@
       <c r="M9" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N9" s="27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
         <v>101</v>
       </c>
@@ -4454,13 +4549,13 @@
         <v>70</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>20</v>
@@ -4483,8 +4578,11 @@
       <c r="M10" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N10" s="27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
         <v>101</v>
       </c>
@@ -4495,13 +4593,13 @@
         <v>80</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>20</v>
@@ -4524,8 +4622,11 @@
       <c r="M11" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N11" s="27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>20</v>
       </c>
@@ -4565,8 +4666,11 @@
       <c r="M12" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N12" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
         <v>20</v>
       </c>
@@ -4606,8 +4710,11 @@
       <c r="M13" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N13" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
         <v>20</v>
       </c>
@@ -4647,8 +4754,11 @@
       <c r="M14" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N14" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
         <v>20</v>
       </c>
@@ -4688,8 +4798,11 @@
       <c r="M15" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N15" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
         <v>20</v>
       </c>
@@ -4729,8 +4842,11 @@
       <c r="M16" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N16" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
         <v>20</v>
       </c>
@@ -4770,8 +4886,11 @@
       <c r="M17" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N17" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
         <v>20</v>
       </c>
@@ -4811,8 +4930,11 @@
       <c r="M18" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N18" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
         <v>20</v>
       </c>
@@ -4852,8 +4974,11 @@
       <c r="M19" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N19" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
         <v>20</v>
       </c>
@@ -4893,8 +5018,11 @@
       <c r="M20" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N20" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
         <v>20</v>
       </c>
@@ -4934,8 +5062,11 @@
       <c r="M21" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N21" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
         <v>20</v>
       </c>
@@ -4975,8 +5106,11 @@
       <c r="M22" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N22" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="27" t="s">
         <v>20</v>
       </c>
@@ -5016,8 +5150,11 @@
       <c r="M23" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N23" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
         <v>20</v>
       </c>
@@ -5057,8 +5194,11 @@
       <c r="M24" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N24" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="27" t="s">
         <v>20</v>
       </c>
@@ -5098,8 +5238,11 @@
       <c r="M25" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N25" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="27" t="s">
         <v>20</v>
       </c>
@@ -5139,8 +5282,11 @@
       <c r="M26" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N26" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="27" t="s">
         <v>20</v>
       </c>
@@ -5180,8 +5326,11 @@
       <c r="M27" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N27" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="27" t="s">
         <v>20</v>
       </c>
@@ -5221,8 +5370,11 @@
       <c r="M28" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N28" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="27" t="s">
         <v>20</v>
       </c>
@@ -5262,8 +5414,11 @@
       <c r="M29" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N29" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="27" t="s">
         <v>20</v>
       </c>
@@ -5303,8 +5458,11 @@
       <c r="M30" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N30" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="27" t="s">
         <v>20</v>
       </c>
@@ -5344,8 +5502,11 @@
       <c r="M31" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N31" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="27" t="s">
         <v>20</v>
       </c>
@@ -5385,8 +5546,11 @@
       <c r="M32" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N32" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="27" t="s">
         <v>20</v>
       </c>
@@ -5426,8 +5590,11 @@
       <c r="M33" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N33" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="27" t="s">
         <v>20</v>
       </c>
@@ -5467,8 +5634,11 @@
       <c r="M34" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N34" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="27" t="s">
         <v>20</v>
       </c>
@@ -5508,8 +5678,11 @@
       <c r="M35" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N35" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="27" t="s">
         <v>20</v>
       </c>
@@ -5549,8 +5722,11 @@
       <c r="M36" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N36" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="27" t="s">
         <v>20</v>
       </c>
@@ -5590,8 +5766,11 @@
       <c r="M37" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N37" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="27" t="s">
         <v>20</v>
       </c>
@@ -5631,8 +5810,11 @@
       <c r="M38" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N38" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="27" t="s">
         <v>20</v>
       </c>
@@ -5672,8 +5854,11 @@
       <c r="M39" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N39" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="27" t="s">
         <v>20</v>
       </c>
@@ -5713,8 +5898,11 @@
       <c r="M40" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N40" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="27" t="s">
         <v>20</v>
       </c>
@@ -5754,8 +5942,11 @@
       <c r="M41" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N41" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="27" t="s">
         <v>20</v>
       </c>
@@ -5795,8 +5986,11 @@
       <c r="M42" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N42" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="27" t="s">
         <v>20</v>
       </c>
@@ -5836,8 +6030,11 @@
       <c r="M43" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N43" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="27" t="s">
         <v>20</v>
       </c>
@@ -5877,8 +6074,11 @@
       <c r="M44" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N44" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="27" t="s">
         <v>20</v>
       </c>
@@ -5918,8 +6118,11 @@
       <c r="M45" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N45" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="27" t="s">
         <v>20</v>
       </c>
@@ -5959,8 +6162,11 @@
       <c r="M46" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N46" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="27" t="s">
         <v>20</v>
       </c>
@@ -6000,8 +6206,11 @@
       <c r="M47" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N47" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="27" t="s">
         <v>20</v>
       </c>
@@ -6041,8 +6250,11 @@
       <c r="M48" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N48" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="27" t="s">
         <v>20</v>
       </c>
@@ -6082,8 +6294,11 @@
       <c r="M49" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N49" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="27" t="s">
         <v>20</v>
       </c>
@@ -6123,8 +6338,11 @@
       <c r="M50" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N50" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="27" t="s">
         <v>20</v>
       </c>
@@ -6164,8 +6382,11 @@
       <c r="M51" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N51" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="27" t="s">
         <v>20</v>
       </c>
@@ -6205,8 +6426,11 @@
       <c r="M52" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N52" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="27" t="s">
         <v>20</v>
       </c>
@@ -6246,8 +6470,11 @@
       <c r="M53" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N53" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>20</v>
       </c>
@@ -6287,8 +6514,11 @@
       <c r="M54" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N54" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="27" t="s">
         <v>20</v>
       </c>
@@ -6328,8 +6558,11 @@
       <c r="M55" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N55" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="27" t="s">
         <v>20</v>
       </c>
@@ -6369,8 +6602,11 @@
       <c r="M56" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N56" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="27" t="s">
         <v>20</v>
       </c>
@@ -6410,8 +6646,11 @@
       <c r="M57" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N57" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="27" t="s">
         <v>20</v>
       </c>
@@ -6451,8 +6690,11 @@
       <c r="M58" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N58" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="27" t="s">
         <v>20</v>
       </c>
@@ -6492,8 +6734,11 @@
       <c r="M59" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N59" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" s="27" t="s">
         <v>20</v>
       </c>
@@ -6533,8 +6778,11 @@
       <c r="M60" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N60" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="27" t="s">
         <v>20</v>
       </c>
@@ -6574,8 +6822,11 @@
       <c r="M61" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N61" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="27" t="s">
         <v>20</v>
       </c>
@@ -6615,8 +6866,11 @@
       <c r="M62" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N62" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" s="27" t="s">
         <v>20</v>
       </c>
@@ -6656,8 +6910,11 @@
       <c r="M63" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N63" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="27" t="s">
         <v>20</v>
       </c>
@@ -6697,8 +6954,11 @@
       <c r="M64" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N64" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="27" t="s">
         <v>20</v>
       </c>
@@ -6738,8 +6998,11 @@
       <c r="M65" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N65" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="27" t="s">
         <v>20</v>
       </c>
@@ -6779,8 +7042,11 @@
       <c r="M66" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N66" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" s="27" t="s">
         <v>20</v>
       </c>
@@ -6820,8 +7086,11 @@
       <c r="M67" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N67" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="27" t="s">
         <v>20</v>
       </c>
@@ -6861,8 +7130,11 @@
       <c r="M68" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N68" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" s="27" t="s">
         <v>20</v>
       </c>
@@ -6902,8 +7174,11 @@
       <c r="M69" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N69" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="27" t="s">
         <v>20</v>
       </c>
@@ -6943,8 +7218,11 @@
       <c r="M70" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N70" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" s="27" t="s">
         <v>20</v>
       </c>
@@ -6984,8 +7262,11 @@
       <c r="M71" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N71" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="27" t="s">
         <v>20</v>
       </c>
@@ -7025,8 +7306,11 @@
       <c r="M72" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N72" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="27" t="s">
         <v>20</v>
       </c>
@@ -7066,8 +7350,11 @@
       <c r="M73" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N73" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74" s="27" t="s">
         <v>20</v>
       </c>
@@ -7107,8 +7394,11 @@
       <c r="M74" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N74" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" s="27" t="s">
         <v>20</v>
       </c>
@@ -7148,8 +7438,11 @@
       <c r="M75" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N75" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" s="27" t="s">
         <v>20</v>
       </c>
@@ -7189,8 +7482,11 @@
       <c r="M76" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N76" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77" s="27" t="s">
         <v>20</v>
       </c>
@@ -7230,8 +7526,11 @@
       <c r="M77" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N77" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78" s="27" t="s">
         <v>20</v>
       </c>
@@ -7271,8 +7570,11 @@
       <c r="M78" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N78" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" s="27" t="s">
         <v>20</v>
       </c>
@@ -7312,8 +7614,11 @@
       <c r="M79" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N79" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" s="27" t="s">
         <v>20</v>
       </c>
@@ -7353,8 +7658,11 @@
       <c r="M80" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N80" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A81" s="27" t="s">
         <v>20</v>
       </c>
@@ -7394,8 +7702,11 @@
       <c r="M81" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N81" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82" s="27" t="s">
         <v>20</v>
       </c>
@@ -7435,8 +7746,11 @@
       <c r="M82" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N82" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A83" s="27" t="s">
         <v>20</v>
       </c>
@@ -7476,8 +7790,11 @@
       <c r="M83" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N83" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A84" s="27" t="s">
         <v>20</v>
       </c>
@@ -7517,8 +7834,11 @@
       <c r="M84" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N84" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A85" s="27" t="s">
         <v>20</v>
       </c>
@@ -7558,8 +7878,11 @@
       <c r="M85" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N85" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="27" t="s">
         <v>20</v>
       </c>
@@ -7599,8 +7922,11 @@
       <c r="M86" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N86" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" s="27" t="s">
         <v>20</v>
       </c>
@@ -7640,8 +7966,11 @@
       <c r="M87" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N87" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="27" t="s">
         <v>20</v>
       </c>
@@ -7681,8 +8010,11 @@
       <c r="M88" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N88" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" s="27" t="s">
         <v>20</v>
       </c>
@@ -7722,8 +8054,11 @@
       <c r="M89" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N89" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A90" s="27" t="s">
         <v>20</v>
       </c>
@@ -7763,8 +8098,11 @@
       <c r="M90" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N90" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A91" s="27" t="s">
         <v>20</v>
       </c>
@@ -7804,8 +8142,11 @@
       <c r="M91" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N91" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A92" s="27" t="s">
         <v>20</v>
       </c>
@@ -7845,8 +8186,11 @@
       <c r="M92" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N92" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93" s="27" t="s">
         <v>20</v>
       </c>
@@ -7886,8 +8230,11 @@
       <c r="M93" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N93" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94" s="27" t="s">
         <v>20</v>
       </c>
@@ -7927,8 +8274,11 @@
       <c r="M94" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N94" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95" s="27" t="s">
         <v>20</v>
       </c>
@@ -7968,8 +8318,11 @@
       <c r="M95" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N95" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A96" s="27" t="s">
         <v>20</v>
       </c>
@@ -8009,8 +8362,11 @@
       <c r="M96" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N96" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A97" s="27" t="s">
         <v>20</v>
       </c>
@@ -8050,8 +8406,11 @@
       <c r="M97" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N97" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98" s="27" t="s">
         <v>20</v>
       </c>
@@ -8091,8 +8450,11 @@
       <c r="M98" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N98" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="27" t="s">
         <v>20</v>
       </c>
@@ -8132,8 +8494,11 @@
       <c r="M99" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N99" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100" s="27" t="s">
         <v>20</v>
       </c>
@@ -8173,8 +8538,11 @@
       <c r="M100" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N100" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A101" s="27" t="s">
         <v>20</v>
       </c>
@@ -8214,8 +8582,11 @@
       <c r="M101" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N101" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A102" s="27" t="s">
         <v>20</v>
       </c>
@@ -8255,8 +8626,11 @@
       <c r="M102" s="27" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N102" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A103" s="27" t="s">
         <v>20</v>
       </c>
@@ -8294,6 +8668,9 @@
         <v>20</v>
       </c>
       <c r="M103" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="N103" s="27" t="s">
         <v>20</v>
       </c>
     </row>
@@ -8352,7 +8729,7 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8375,10 +8752,10 @@
     </row>
     <row r="2" spans="7:17" x14ac:dyDescent="0.25">
       <c r="G2" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J2" s="30" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K2" s="31">
         <f>ROUND('02_Capacity'!$E$27,1)</f>
@@ -8393,16 +8770,16 @@
         <f>ROUND('02_Capacity'!$E$30,1)</f>
       </c>
       <c r="P2" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="7:17" x14ac:dyDescent="0.25">
       <c r="G3" s="1"/>
       <c r="J3" s="30" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="K3" s="31">
         <f>ROUND((SUMIFS(tblPlanActive[AN],tblPlanActive[Статус на конец квартала],"&lt;&gt;Отложено"))*(1+IFERROR(IF(AND(ISNUMBER('99_Справочники'!$C$35),'99_Справочники'!$C$35&gt;=0,'99_Справочники'!$C$35&lt;=1),'99_Справочники'!$C$35,0.2),0.2)),1)</f>
@@ -8422,7 +8799,7 @@
     <row r="4" spans="7:17" x14ac:dyDescent="0.25">
       <c r="G4" s="1"/>
       <c r="J4" s="30" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K4" s="31">
         <f>ROUND('02_Capacity'!$E$27-(SUMIFS(tblPlanActive[AN],tblPlanActive[Статус на конец квартала],"&lt;&gt;Отложено"))*(1+IFERROR(IF(AND(ISNUMBER('99_Справочники'!$C$35),'99_Справочники'!$C$35&gt;=0,'99_Справочники'!$C$35&lt;=1),'99_Справочники'!$C$35,0.2),0.2)),1)</f>
@@ -8441,7 +8818,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" s="32" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B5" s="32" t="s">
         <v>145</v>
@@ -10002,7 +10379,7 @@
     </row>
     <row r="30" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A30" s="32" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B30" s="32" t="s">
         <v>145</v>
@@ -11568,7 +11945,7 @@
     </row>
     <row r="55" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A55" s="32" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B55" s="32" t="s">
         <v>145</v>
@@ -11666,7 +12043,7 @@
     </row>
     <row r="56" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A56" s="33" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B56" s="33" t="s">
         <v>20</v>
@@ -11684,16 +12061,16 @@
         <v>10</v>
       </c>
       <c r="G56" s="35" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H56" s="35" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I56" s="35" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J56" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K56" s="36">
         <v>3</v>
@@ -11738,7 +12115,7 @@
     </row>
     <row r="57" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A57" s="33" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B57" s="33" t="s">
         <v>20</v>
@@ -11756,13 +12133,13 @@
         <v>20</v>
       </c>
       <c r="G57" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H57" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I57" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J57" s="35" t="s">
         <v>20</v>
@@ -11810,7 +12187,7 @@
     </row>
     <row r="58" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A58" s="33" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B58" s="33" t="s">
         <v>20</v>
@@ -11828,13 +12205,13 @@
         <v>30</v>
       </c>
       <c r="G58" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H58" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I58" s="35" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J58" s="35" t="s">
         <v>20</v>
@@ -11882,7 +12259,7 @@
     </row>
     <row r="59" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A59" s="33" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B59" s="33" t="s">
         <v>20</v>
@@ -11900,13 +12277,13 @@
         <v>40</v>
       </c>
       <c r="G59" s="35" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H59" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I59" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J59" s="35" t="s">
         <v>20</v>
@@ -11954,7 +12331,7 @@
     </row>
     <row r="60" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A60" s="33" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B60" s="33" t="s">
         <v>20</v>
@@ -11972,13 +12349,13 @@
         <v>50</v>
       </c>
       <c r="G60" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H60" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I60" s="35" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J60" s="35" t="s">
         <v>20</v>
@@ -12026,7 +12403,7 @@
     </row>
     <row r="61" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A61" s="33" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B61" s="33" t="s">
         <v>20</v>
@@ -12044,13 +12421,13 @@
         <v>60</v>
       </c>
       <c r="G61" s="35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H61" s="35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I61" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J61" s="35" t="s">
         <v>20</v>
@@ -12098,7 +12475,7 @@
     </row>
     <row r="62" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A62" s="33" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B62" s="33" t="s">
         <v>20</v>
@@ -12116,13 +12493,13 @@
         <v>70</v>
       </c>
       <c r="G62" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H62" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I62" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J62" s="35" t="s">
         <v>20</v>
@@ -12170,7 +12547,7 @@
     </row>
     <row r="63" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A63" s="33" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B63" s="33" t="s">
         <v>20</v>
@@ -12188,13 +12565,13 @@
         <v>80</v>
       </c>
       <c r="G63" s="35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H63" s="35" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I63" s="35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J63" s="35" t="s">
         <v>20</v>
@@ -21366,4 +21743,99 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="36.42857142857143" customWidth="1"/>
+    <col min="2" max="2" width="4.285714285714286" customWidth="1"/>
+    <col min="3" max="3" width="36.42857142857143" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="8" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C8" s="4" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="9" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="10" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C10" s="4" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="11" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C11" s="4" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="12" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C12" s="4" t="s">
+        <v>295</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add JQL and task comment actions
</commit_message>
<xml_diff>
--- a/outputs/quarter_planning_step1.xlsx
+++ b/outputs/quarter_planning_step1.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4713" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4717" uniqueCount="297">
   <si>
     <t>Настройки квартального планирования</t>
   </si>
@@ -321,6 +321,9 @@
   </si>
   <si>
     <t>Импорт CSV (до 100)</t>
+  </si>
+  <si>
+    <t>JQL</t>
   </si>
   <si>
     <t>&gt;</t>
@@ -4217,6 +4220,9 @@
       <c r="D2" s="27" t="s">
         <v>100</v>
       </c>
+      <c r="F2" s="27" t="s">
+        <v>101</v>
+      </c>
       <c r="H2" s="28">
         <f>SUM(H4:H103)</f>
       </c>
@@ -4232,37 +4238,37 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>3</v>
@@ -4271,12 +4277,12 @@
         <v>94</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B4" s="27" t="s">
         <v>20</v>
@@ -4285,16 +4291,16 @@
         <v>10</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H4" s="29">
         <v>3</v>
@@ -4315,12 +4321,12 @@
         <v>20</v>
       </c>
       <c r="N4" s="27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B5" s="27" t="s">
         <v>20</v>
@@ -4329,13 +4335,13 @@
         <v>20</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>20</v>
@@ -4359,12 +4365,12 @@
         <v>20</v>
       </c>
       <c r="N5" s="27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B6" s="27" t="s">
         <v>20</v>
@@ -4373,13 +4379,13 @@
         <v>30</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>20</v>
@@ -4403,12 +4409,12 @@
         <v>20</v>
       </c>
       <c r="N6" s="27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B7" s="27" t="s">
         <v>20</v>
@@ -4417,13 +4423,13 @@
         <v>40</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>20</v>
@@ -4447,12 +4453,12 @@
         <v>20</v>
       </c>
       <c r="N7" s="27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B8" s="27" t="s">
         <v>20</v>
@@ -4461,13 +4467,13 @@
         <v>50</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>20</v>
@@ -4491,12 +4497,12 @@
         <v>20</v>
       </c>
       <c r="N8" s="27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B9" s="27" t="s">
         <v>20</v>
@@ -4505,13 +4511,13 @@
         <v>60</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>20</v>
@@ -4535,12 +4541,12 @@
         <v>20</v>
       </c>
       <c r="N9" s="27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B10" s="27" t="s">
         <v>20</v>
@@ -4549,13 +4555,13 @@
         <v>70</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>20</v>
@@ -4579,12 +4585,12 @@
         <v>20</v>
       </c>
       <c r="N10" s="27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B11" s="27" t="s">
         <v>20</v>
@@ -4593,13 +4599,13 @@
         <v>80</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>20</v>
@@ -4623,7 +4629,7 @@
         <v>20</v>
       </c>
       <c r="N11" s="27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -8729,7 +8735,7 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8752,10 +8758,10 @@
     </row>
     <row r="2" spans="7:17" x14ac:dyDescent="0.25">
       <c r="G2" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J2" s="30" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K2" s="31">
         <f>ROUND('02_Capacity'!$E$27,1)</f>
@@ -8770,16 +8776,16 @@
         <f>ROUND('02_Capacity'!$E$30,1)</f>
       </c>
       <c r="P2" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="7:17" x14ac:dyDescent="0.25">
       <c r="G3" s="1"/>
       <c r="J3" s="30" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K3" s="31">
         <f>ROUND((SUMIFS(tblPlanActive[AN],tblPlanActive[Статус на конец квартала],"&lt;&gt;Отложено"))*(1+IFERROR(IF(AND(ISNUMBER('99_Справочники'!$C$35),'99_Справочники'!$C$35&gt;=0,'99_Справочники'!$C$35&lt;=1),'99_Справочники'!$C$35,0.2),0.2)),1)</f>
@@ -8798,8 +8804,11 @@
     </row>
     <row r="4" spans="7:17" x14ac:dyDescent="0.25">
       <c r="G4" s="1"/>
+      <c r="I4" s="27" t="s">
+        <v>101</v>
+      </c>
       <c r="J4" s="30" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K4" s="31">
         <f>ROUND('02_Capacity'!$E$27-(SUMIFS(tblPlanActive[AN],tblPlanActive[Статус на конец квартала],"&lt;&gt;Отложено"))*(1+IFERROR(IF(AND(ISNUMBER('99_Справочники'!$C$35),'99_Справочники'!$C$35&gt;=0,'99_Справочники'!$C$35&lt;=1),'99_Справочники'!$C$35,0.2),0.2)),1)</f>
@@ -8818,100 +8827,100 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="D5" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>149</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="N5" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B5" s="32" t="s">
-        <v>145</v>
-      </c>
-      <c r="C5" s="32" t="s">
-        <v>146</v>
-      </c>
-      <c r="D5" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="E5" s="32" t="s">
-        <v>148</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="O5" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="S5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="U5" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="V5" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="W5" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="X5" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="Y5" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="Z5" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AA5" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AB5" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AC5" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="AD5" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AE5" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AF5" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.25">
@@ -10356,7 +10365,7 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B28" s="39"/>
       <c r="C28" s="39"/>
@@ -10377,102 +10386,107 @@
       <c r="R28" s="39"/>
       <c r="S28" s="39"/>
     </row>
+    <row r="29" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I29" s="27" t="s">
+        <v>101</v>
+      </c>
+    </row>
     <row r="30" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A30" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="B30" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C30" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="D30" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="E30" s="32" t="s">
+        <v>149</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="M30" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="N30" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B30" s="32" t="s">
-        <v>145</v>
-      </c>
-      <c r="C30" s="32" t="s">
-        <v>146</v>
-      </c>
-      <c r="D30" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="E30" s="32" t="s">
-        <v>148</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="M30" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="N30" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="O30" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P30" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="Q30" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R30" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="S30" s="2" t="s">
         <v>3</v>
       </c>
       <c r="T30" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="U30" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="V30" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="W30" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="X30" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="Y30" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="Z30" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AA30" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AB30" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AC30" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="AD30" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AE30" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AF30" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="31" spans="1:32" x14ac:dyDescent="0.25">
@@ -11917,7 +11931,7 @@
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -11938,112 +11952,115 @@
       <c r="R53" s="1"/>
       <c r="S53" s="1"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
+      </c>
+      <c r="I54" s="27" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="55" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A55" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="B55" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C55" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="D55" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="E55" s="32" t="s">
+        <v>149</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="M55" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="N55" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B55" s="32" t="s">
-        <v>145</v>
-      </c>
-      <c r="C55" s="32" t="s">
-        <v>146</v>
-      </c>
-      <c r="D55" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="E55" s="32" t="s">
-        <v>148</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="H55" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="I55" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="J55" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="K55" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="L55" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="M55" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="N55" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="O55" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P55" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="Q55" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R55" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="S55" s="2" t="s">
         <v>3</v>
       </c>
       <c r="T55" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="U55" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="V55" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="W55" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="X55" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="Y55" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="Z55" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AA55" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="AB55" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AC55" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="AD55" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AE55" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AF55" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="56" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A56" s="33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B56" s="33" t="s">
         <v>20</v>
@@ -12061,16 +12078,16 @@
         <v>10</v>
       </c>
       <c r="G56" s="35" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H56" s="35" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I56" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J56" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K56" s="36">
         <v>3</v>
@@ -12115,7 +12132,7 @@
     </row>
     <row r="57" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A57" s="33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B57" s="33" t="s">
         <v>20</v>
@@ -12133,13 +12150,13 @@
         <v>20</v>
       </c>
       <c r="G57" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H57" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I57" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J57" s="35" t="s">
         <v>20</v>
@@ -12187,7 +12204,7 @@
     </row>
     <row r="58" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A58" s="33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B58" s="33" t="s">
         <v>20</v>
@@ -12205,13 +12222,13 @@
         <v>30</v>
       </c>
       <c r="G58" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H58" s="35" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I58" s="35" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J58" s="35" t="s">
         <v>20</v>
@@ -12259,7 +12276,7 @@
     </row>
     <row r="59" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A59" s="33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B59" s="33" t="s">
         <v>20</v>
@@ -12277,13 +12294,13 @@
         <v>40</v>
       </c>
       <c r="G59" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H59" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I59" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J59" s="35" t="s">
         <v>20</v>
@@ -12331,7 +12348,7 @@
     </row>
     <row r="60" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A60" s="33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B60" s="33" t="s">
         <v>20</v>
@@ -12349,13 +12366,13 @@
         <v>50</v>
       </c>
       <c r="G60" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H60" s="35" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I60" s="35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J60" s="35" t="s">
         <v>20</v>
@@ -12403,7 +12420,7 @@
     </row>
     <row r="61" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A61" s="33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B61" s="33" t="s">
         <v>20</v>
@@ -12421,13 +12438,13 @@
         <v>60</v>
       </c>
       <c r="G61" s="35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H61" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I61" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J61" s="35" t="s">
         <v>20</v>
@@ -12475,7 +12492,7 @@
     </row>
     <row r="62" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A62" s="33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B62" s="33" t="s">
         <v>20</v>
@@ -12493,13 +12510,13 @@
         <v>70</v>
       </c>
       <c r="G62" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H62" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I62" s="35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J62" s="35" t="s">
         <v>20</v>
@@ -12547,7 +12564,7 @@
     </row>
     <row r="63" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A63" s="33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B63" s="33" t="s">
         <v>20</v>
@@ -12565,13 +12582,13 @@
         <v>80</v>
       </c>
       <c r="G63" s="35" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H63" s="35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I63" s="35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J63" s="35" t="s">
         <v>20</v>
@@ -19423,7 +19440,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -19431,102 +19448,102 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C4" s="3">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C5" s="3">
         <v>2</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C6" s="3">
         <v>3</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C7" s="3">
         <v>4</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E8" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E9" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E10" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -19537,10 +19554,10 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -19550,10 +19567,10 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -19563,10 +19580,10 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -19576,10 +19593,10 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -19589,10 +19606,10 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -19602,10 +19619,10 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -19615,10 +19632,10 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -19628,10 +19645,10 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
@@ -19641,10 +19658,10 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
@@ -19654,10 +19671,10 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
@@ -19667,10 +19684,10 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
@@ -19680,10 +19697,10 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
@@ -19693,10 +19710,10 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
@@ -19706,10 +19723,10 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
@@ -19719,10 +19736,10 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -19732,121 +19749,121 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C30" s="40">
         <v>5</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C31" s="41">
         <v>0.5</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C32" s="40">
         <v>5</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C33" s="41">
         <v>0.5</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C34" s="41">
         <v>0.5</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C35" s="41">
         <v>0.2</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -19913,7 +19930,7 @@
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="42" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B1" s="42"/>
       <c r="C1" s="42"/>
@@ -19929,7 +19946,7 @@
         <v>20</v>
       </c>
       <c r="M1" s="44" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="N1" s="44" t="s">
         <v>20</v>
@@ -19973,7 +19990,7 @@
         <v>20</v>
       </c>
       <c r="D2" s="47" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E2" s="48" t="s">
         <v>20</v>
@@ -19988,10 +20005,10 @@
         <v>20</v>
       </c>
       <c r="M2" s="47" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="N2" s="49" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="O2" s="49"/>
       <c r="P2" s="49"/>
@@ -20026,7 +20043,7 @@
         <v>20</v>
       </c>
       <c r="D3" s="44" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E3" s="51" t="s">
         <v>20</v>
@@ -20041,10 +20058,10 @@
         <v>20</v>
       </c>
       <c r="M3" s="44" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="N3" s="52" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="O3" s="52"/>
       <c r="P3" s="52"/>
@@ -20079,7 +20096,7 @@
         <v>20</v>
       </c>
       <c r="D4" s="47" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E4" s="48" t="s">
         <v>20</v>
@@ -20094,10 +20111,10 @@
         <v>20</v>
       </c>
       <c r="M4" s="47" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="N4" s="49" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="O4" s="49"/>
       <c r="P4" s="49"/>
@@ -20132,7 +20149,7 @@
         <v>20</v>
       </c>
       <c r="D5" s="44" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>20</v>
@@ -20147,10 +20164,10 @@
         <v>20</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="N5" s="52" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O5" s="52"/>
       <c r="P5" s="52"/>
@@ -20185,7 +20202,7 @@
         <v>20</v>
       </c>
       <c r="D6" s="47" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E6" s="48" t="s">
         <v>20</v>
@@ -20200,10 +20217,10 @@
         <v>20</v>
       </c>
       <c r="M6" s="47" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="N6" s="49" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="O6" s="49"/>
       <c r="P6" s="49"/>
@@ -20238,7 +20255,7 @@
         <v>20</v>
       </c>
       <c r="D7" s="44" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E7" s="51" t="s">
         <v>20</v>
@@ -20297,7 +20314,7 @@
         <v>20</v>
       </c>
       <c r="D8" s="47" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E8" s="48" t="s">
         <v>20</v>
@@ -20356,7 +20373,7 @@
         <v>20</v>
       </c>
       <c r="D9" s="44" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E9" s="51" t="s">
         <v>20</v>
@@ -20415,7 +20432,7 @@
         <v>20</v>
       </c>
       <c r="D10" s="47" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E10" s="48" t="s">
         <v>20</v>
@@ -20474,7 +20491,7 @@
         <v>20</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E11" s="51" t="s">
         <v>20</v>
@@ -20533,7 +20550,7 @@
         <v>20</v>
       </c>
       <c r="D12" s="47" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E12" s="48" t="s">
         <v>20</v>
@@ -20592,7 +20609,7 @@
         <v>20</v>
       </c>
       <c r="D13" s="44" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E13" s="51" t="s">
         <v>20</v>
@@ -20713,19 +20730,19 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="52" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B15" s="52"/>
       <c r="C15" s="52"/>
       <c r="D15" s="52"/>
       <c r="E15" s="51" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F15" s="51" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G15" s="51" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="H15" s="51"/>
       <c r="I15" s="51"/>
@@ -20744,7 +20761,7 @@
         <v>20</v>
       </c>
       <c r="P15" s="57" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="Q15" s="57" t="s">
         <v>20</v>
@@ -20776,60 +20793,60 @@
       <c r="E16" s="51"/>
       <c r="F16" s="51"/>
       <c r="G16" s="47" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H16" s="47" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I16" s="47" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J16" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="K16" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="L16" s="47" t="s">
+        <v>269</v>
+      </c>
+      <c r="M16" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="N16" s="58" t="s">
+        <v>270</v>
+      </c>
+      <c r="O16" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="P16" s="58" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q16" s="58" t="s">
+        <v>268</v>
+      </c>
+      <c r="R16" s="58" t="s">
         <v>110</v>
       </c>
-      <c r="K16" s="47" t="s">
+      <c r="S16" s="58" t="s">
         <v>111</v>
       </c>
-      <c r="L16" s="47" t="s">
-        <v>268</v>
-      </c>
-      <c r="M16" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="N16" s="58" t="s">
-        <v>269</v>
-      </c>
-      <c r="O16" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="P16" s="58" t="s">
-        <v>174</v>
-      </c>
-      <c r="Q16" s="58" t="s">
-        <v>267</v>
-      </c>
-      <c r="R16" s="58" t="s">
-        <v>109</v>
-      </c>
-      <c r="S16" s="58" t="s">
-        <v>110</v>
-      </c>
       <c r="T16" s="58" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="U16" s="58" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="V16" s="58" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="W16" s="58" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="52" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B17" s="52"/>
       <c r="C17" s="52"/>
@@ -20867,7 +20884,7 @@
         <v>20</v>
       </c>
       <c r="N17" s="57" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="O17" s="43" t="s">
         <v>20</v>
@@ -20907,7 +20924,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="49" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C18" s="49"/>
       <c r="D18" s="49"/>
@@ -20944,7 +20961,7 @@
         <v>20</v>
       </c>
       <c r="N18" s="59" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="O18" s="46" t="s">
         <v>20</v>
@@ -20982,7 +20999,7 @@
         <v>20</v>
       </c>
       <c r="C19" s="49" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D19" s="49"/>
       <c r="E19" s="47" t="s">
@@ -21013,7 +21030,7 @@
         <v>20</v>
       </c>
       <c r="N19" s="46" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O19" s="46" t="s">
         <v>20</v>
@@ -21051,7 +21068,7 @@
         <v>20</v>
       </c>
       <c r="C20" s="52" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D20" s="52"/>
       <c r="E20" s="44" t="s">
@@ -21115,7 +21132,7 @@
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="47"/>
       <c r="B21" s="49" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C21" s="49"/>
       <c r="D21" s="49"/>
@@ -21153,7 +21170,7 @@
         <v>20</v>
       </c>
       <c r="C22" s="49" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D22" s="49"/>
       <c r="E22" s="47" t="s">
@@ -21185,7 +21202,7 @@
         <v>20</v>
       </c>
       <c r="C23" s="52" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D23" s="52"/>
       <c r="E23" s="44" t="s">
@@ -21757,74 +21774,74 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C8" s="4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="9" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C9" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="10" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C10" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="11" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C11" s="4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="12" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C12" s="4" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>